<commit_message>
fix : erreur merge
</commit_message>
<xml_diff>
--- a/Projet Power4 - Gestion de projet - Groupe XX.xlsx
+++ b/Projet Power4 - Gestion de projet - Groupe XX.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thefl\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thefl\Desktop\Ynov 2526\Module - Proj1 HTML CSS\projet-power4-groupe-4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{739E8FE2-EAF8-4B53-802F-A97C24223FC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8F0309A-BC3D-4C8E-BAE2-442B8306902A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2616" yWindow="2616" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2928" yWindow="3720" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="28">
   <si>
     <t>Membre 2</t>
   </si>
@@ -111,6 +111,15 @@
   </si>
   <si>
     <t>Projet Power'4 - Gestion de projet - Groupe 4</t>
+  </si>
+  <si>
+    <t>game-init.go</t>
+  </si>
+  <si>
+    <t>23,10,2025</t>
+  </si>
+  <si>
+    <t>A tester, peut être plus de gestions à faire</t>
   </si>
 </sst>
 </file>
@@ -893,15 +902,25 @@
       <c r="E6" s="21">
         <v>1</v>
       </c>
-      <c r="F6" s="3"/>
-      <c r="G6" s="2"/>
+      <c r="F6" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="H6" s="2"/>
       <c r="I6" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="J6" s="5"/>
-      <c r="K6" s="5"/>
-      <c r="L6" s="13"/>
+        <v>12</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="L6" s="13" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B7" s="23" t="s">

</xml_diff>